<commit_message>
Update bug reports and test case documentation; enhance clarity and detail in defect descriptions
</commit_message>
<xml_diff>
--- a/HW1/R3_device/R3_TestCases_Checklist_Summary.xlsx
+++ b/HW1/R3_device/R3_TestCases_Checklist_Summary.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +53,7 @@
       <b val="1"/>
       <color rgb="001F4E78"/>
     </font>
+    <font/>
   </fonts>
   <fills count="7">
     <fill>
@@ -113,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -147,6 +148,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -513,7 +520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -526,6 +533,7 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -577,6 +585,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Video</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Ước tính</t>
         </is>
       </c>
     </row>
@@ -615,16 +628,25 @@
           <t>Mỗi lần nhấn: phím mới chìm xuống, phím cũ nảy lên hết. Tốc độ tăng dần qua 3 cấp. Nhấn 0 thì động cơ ngắt, cánh giảm tốc theo quán tính rồi dừng. Không rè, không rung bất thường.</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Mỗi lần bấm, phím trước nảy lên và phím mới chìm xuống. Động cơ chạy ở cả 3 cấp, gió tăng dần. Bấm 0 thì phím 3 nảy lên, cánh giảm tốc theo quán tính rồi dừng hẳn, không rè, không rung bất thường.</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Video 1</t>
+          <t>https://youtube.com/shorts/JEd-FkanM2o</t>
+        </is>
+      </c>
+      <c r="K2" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -663,16 +685,25 @@
 Kéo chốt: dừng quét ngay tại vị trí hiện tại, cánh vẫn quay bình thường.</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Khi ấn chốt, đầu quạt quét đều hai bên, không kêu lục cục, không khựng. Khi kéo chốt lên, quạt dừng quét ngay tại vị trí đang đứng và giữ nguyên hướng thổi, cánh vẫn quay bình thường.</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Video 2</t>
+          <t>https://youtube.com/shorts/eEpm26qTveE</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -684,7 +715,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Gemini</t>
+          <t>Gemini (rút gọn)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -694,29 +725,39 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Quạt chạy số 3; lực tay nâng/hạ lồng quạt.</t>
+          <t>Quạt chạy số 3; dùng tay nâng/hạ lồng quạt.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1. Nhấn phím 3.
-2. Đẩy lồng quạt ngửa lên góc tối đa, buông tay, chờ 60s.
-3. Ấn lồng quạt cúi xuống góc tối đa, buông tay, chờ 60s.</t>
+          <t>1. Bật số 3.
+2. Đẩy lồng quạt ngửa lên góc tối đa, buông tay, đếm 30 giây.
+3. Ấn lồng quạt cúi xuống góc tối đa, buông tay, đếm 30 giây.
+4. Quan sát góc có tự trôi không.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Khớp có lực ma sát vừa đủ, chuyển động chắc. Sau khi buông tay, góc giữ nguyên trong 60s, không tự trôi hay gục xuống dưới phản lực gió.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+          <t>Khớp giữ nguyên góc trong 30 giây ở cả hai vị trí, không tự trôi hoặc gục xuống dưới phản lực gió.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Sau khi buông tay, khớp gập giữ nguyên góc ở cả hai vị trí (ngửa hết cỡ và cúi hết cỡ) trong suốt 30 giây quan sát. Không tự trôi, không gục xuống dưới phản lực gió ở số 3.</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="120" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -726,39 +767,49 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Gemini (đã giảm liều: 20s -&gt; 5s)</t>
+          <t>Claude (thay case có rủi ro làm hỏng thêm)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra ly hợp trượt của hộp bánh răng đảo gió khi hành trình quét bị chặn.</t>
+          <t>Kiểm tra nhãn thông số và cảnh báo an toàn còn nguyên vẹn và đọc được, theo yêu cầu ghi nhãn của TCVN 5699-1 (IEC 60335-1).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Quạt chạy số 3, đang quét; giữ lồng quạt bằng tay trong 5 giây.</t>
+          <t>Quạt đã rút điện; quan sát tem trên thân quạt bằng mắt thường ở khoảng cách đọc bình thường.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>1. Bật số 3, ấn tuốc năng cho quạt quét.
-2. Khi đầu quạt đang xoay, giữ nhẹ lồng quạt chặn hành trình ĐÚNG 5 GIÂY.
-3. Thả tay, quan sát tiếp 2 chu kỳ quét.</t>
+          <t>1. Rút điện.
+2. Đọc toàn bộ tem: hãng, công suất, điện áp, cấp cách điện, cấp chống giật, tiêu chuẩn áp dụng, tháng SX.
+3. Kiểm tra tem có bong, mờ, rách, hay bị che khuất không.
+4. Dùng ngón tay chà nhẹ mặt tem 5 lần, xem chữ có bị nhòe không.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ly hợp trượt hoạt động, bánh răng không vỡ. Không có mùi khét, hộp nhông không nóng bất thường. Sau khi thả, quạt quét lại bình thường, không lệch biên độ.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+          <t>Toàn bộ thông tin bắt buộc còn đọc được rõ ràng. Tem bám chắc, không bong góc, chữ không nhòe sau khi chà nhẹ.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Toàn bộ thông tin bắt buộc trên tem còn đọc rõ: hãng SENKO, 220V/50Hz/40W, cấp cách điện E, cấp chống giật điện cấp 0, TCVN 5699-2-80:2007 (IEC 60335-2-80:2005), lô SX 107, tháng SX 07-2022. Chà nhẹ mặt tem 5 lần, chữ không nhòe. Tem bám chắc, không bong góc, không bị che khuất.</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="120" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -773,37 +824,47 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Đo độ ồn ở từng cấp gió để phát hiện tiếng cơ khí bất thường và kiểm tra mức ồn có tăng hợp lý theo cấp không.</t>
+          <t>Phát hiện tiếng cơ khí bất thường và xác nhận độ ồn tăng hợp lý theo từng cấp gió.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>App đo dB trên điện thoại, đặt cách quạt 1m ngang tầm bầu quạt; phòng yên tĩnh.</t>
+          <t>Phòng yên tĩnh; đứng cách quạt 1m; có thể dùng app đo dB trên điện thoại nếu có.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>1. Đo độ ồn nền của phòng khi quạt tắt, ghi lại.
-2. Bật số 1, chờ 30s, đo 10s lấy giá trị trung bình.
-3. Lặp lại với số 2 và số 3.
-4. Nghe kỹ tiếng lạch cạch, rít hoặc va đập theo nhịp.</t>
+          <t>1. Quạt tắt: nghe độ ồn nền của phòng.
+2. Bật số 1, nghe 20 giây.
+3. Bật số 2, nghe 20 giây.
+4. Bật số 3, nghe 20 giây.
+5. Chú ý tiếng lạch cạch theo nhịp, tiếng rít kim loại, tiếng va đập từ hộp tuốc năng.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Độ ồn tăng dần theo cấp và cao hơn nền phòng. Không có tiếng lạch cạch theo nhịp, không tiếng rít kim loại, không tiếng va đập từ hộp tuốc năng.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+          <t>Độ ồn tăng dần theo cấp. Chỉ có tiếng gió và tiếng động cơ đều, không có tiếng lạch cạch theo nhịp, không rít, không va đập.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Đánh giá bằng tai, không dùng thiết bị đo. Độ ồn tăng dần qua ba cấp, cấp 3 ồn nhất. Chỉ nghe thấy tiếng gió và tiếng động cơ đều; không có tiếng lạch cạch theo nhịp, không tiếng rít kim loại, không tiếng va đập từ hộp tuốc năng.</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Video 5</t>
+          <t>Video 6 (dự phòng)</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -820,7 +881,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Xác minh động cơ khởi động lại an toàn khi mất điện và có điện lại đột ngột trong lúc công tắc vẫn ở vị trí bật.</t>
+          <t>Xác minh động cơ khởi động lại an toàn khi mất điện rồi có điện lại trong lúc công tắc vẫn ở vị trí bật.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -830,7 +891,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1. Bật quạt số 3, chạy ổn định 30s.
+          <t>1. Bật số 3, chạy ổn định 30 giây.
 2. Rút phích khỏi ổ điện.
 3. Đếm 3 giây.
 4. Cắm lại phích trong khi phím 3 vẫn chìm.</t>
@@ -838,17 +899,26 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Không phát tia lửa lớn tại chân phích. Động cơ khởi động lại êm, cánh đạt lại tốc độ định mức, không kẹt rotor, không có tiếng ù kéo dài.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+          <t>Không có tia lửa lớn tại chân phích. Động cơ khởi động lại êm, cánh đạt lại tốc độ bình thường, không kẹt rotor, không ù kéo dài.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Không quan sát thấy tia lửa tại chân phích khi cắm lại. Động cơ khởi động lại ngay, cánh đạt lại tốc độ bình thường, không kẹt rotor, không có tiếng ù kéo dài.</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="120" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -868,7 +938,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Dải giấy mỏng treo cố định cách mặt lồng quạt 50cm, ngang tâm trục.</t>
+          <t>Tờ giấy mỏng treo cố định trước quạt (ghi rõ khoảng cách thực tế đã dùng khi chạy).</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -884,16 +954,25 @@
           <t>Góc bay của dải giấy tăng rõ rệt qua từng cấp. Không có hai cấp nào cho góc bay gần như bằng nhau.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Độ bay của tờ giấy tăng rõ rệt qua từng cấp: cấp 1 giấy lay nhẹ, cấp 2 bay mạnh hơn, cấp 3 bay mạnh nhất. Ba cấp phân biệt được bằng mắt thường, không có hai cấp nào cho kết quả giống nhau.</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Video 3</t>
+          <t>https://youtube.com/shorts/WYQW7PdwYas</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -933,7 +1012,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Quạt tắt hẳn thay vì chuyển cấp; phím 1 nảy lên nhưng phím 2 không khóa được vị trí.</t>
+          <t>Quạt không nhận cấp tốc độ nào. Cả hai phím đều nảy lên vị trí ngắt, động cơ mất điện và dừng hẳn. Phải bấm lại một lần nữa quạt mới chạy. Tái hiện 3/3 lần. Ngưỡng quan sát: bấm cách nhau từ 0,5 giây trở lên thì chuyển cấp bình thường, nhanh hơn thì quạt tắt.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -948,7 +1027,12 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Video 4</t>
+          <t>https://youtube.com/shorts/HPpBDBBYLWI</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -997,6 +1081,11 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -1044,6 +1133,11 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1091,6 +1185,11 @@
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="120" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -1143,7 +1242,12 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Video 5</t>
+          <t>Anh (khong quay video)</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -1165,14 +1269,15 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Quạt chạy số 2, đang quét; bẻ ngang đầu quạt vượt quá điểm cuối hành trình rồi thả.</t>
+          <t>Quạt chạy số 1, đang quét; dùng tay đẩy đầu quạt sang phải vượt quá điểm cuối hành trình.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>1. Bật số 2, ấn tuốc năng, đánh dấu hai điểm cuối hành trình trên tường.
-2. Bẻ nhẹ đầu quạt vượt quá điểm cuối khoảng 15 độ rồi thả tay.
-3. Theo dõi 3 chu kỳ quét tiếp theo, đo lại biên độ.</t>
+          <t>1. Bật số 1, ấn chốt tuốc năng, để quạt quét ổn định 2 chu kỳ.
+2. Đánh dấu 2 điểm cuối hành trình làm mốc.
+3. Khi đầu quạt đang quét, đẩy mạnh đầu quạt sang phải vượt quá điểm cuối hành trình.
+4. Thả tay, để quạt quét tiếp 2 chu kỳ rồi so với 2 mốc ban đầu.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1182,7 +1287,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Biên độ quét sau khi bẻ bị lệch so với vạch đánh dấu ban đầu, không tự phục hồi.</t>
+          <t>Cánh vẫn quay bình thường nhưng hành trình quét bị dịch hẳn sang một bên; hai điểm cuối không còn trùng mốc ban đầu. Quạt không tự phục hồi dù chạy tiếp, phải tắt và chỉnh lại bằng tay. Tái hiện 2/2 lần.</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1197,7 +1302,12 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Video 4</t>
+          <t>https://youtube.com/shorts/Dtg48KkCVdo</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
         </is>
       </c>
     </row>
@@ -1214,32 +1324,35 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra tính toàn vẹn của dây nguồn, phích cắm và cơ cấu giữ dây tại điểm vào thân quạt, theo yêu cầu an toàn chung TCVN 5699-1 (IEC 60335-1).</t>
+          <t>Kiểm tra tính toàn vẹn của dây nguồn, phích cắm và cơ cấu giữ dây — đặc biệt quan trọng vì quạt thuộc cấp chống giật điện cấp 0, không có tiếp địa bảo vệ.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Quạt đã RÚT ĐIỆN; quan sát bằng mắt và kéo nhẹ bằng tay, không dùng dụng cụ.</t>
+          <t>Quạt đã RÚT ĐIỆN; quan sát bằng mắt và kéo nhẹ bằng tay.</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>1. Rút phích điện.
-2. Vuốt dọc toàn bộ chiều dài dây, tìm vết nứt, chai cứng, gập gãy, cháy xém.
+2. Vuốt dọc toàn bộ dây, tìm vết nứt, chai cứng, gập gãy, cháy xém.
 3. Kiểm tra chân phích: thẳng hay cong, chắc hay lỏng, có gỉ không.
-4. Một tay giữ thân quạt, tay kia kéo nhẹ dây tại điểm vào thân, quan sát dây có xê dịch không.
-5. Kiểm tra điểm nối dây với công tắc nếu nhìn thấy được.</t>
+4. Một tay giữ thân quạt, tay kia kéo nhẹ dây tại điểm vào thân, xem dây có xê dịch không.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Vỏ cách điện liền lạc trên toàn bộ chiều dài, không nứt, không chai, không cháy. Chân phích thẳng và chắc. Dây không xê dịch tại điểm vào thân, không lộ lõi đồng, cơ cấu giữ dây còn tác dụng.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+          <t>Vỏ cách điện liền lạc, không nứt, không chai, không cháy. Chân phích thẳng và chắc. Dây không xê dịch tại điểm vào thân, không lộ lõi đồng.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Vỏ cách điện liền lạc trên toàn bộ chiều dài dây, không nứt, không chai cứng, không cháy xém. Chân phích thẳng và chắc, không gỉ. Kéo nhẹ dây tại điểm vào thân quạt, dây không xê dịch, không lộ lõi đồng.</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1248,6 +1361,11 @@
           <t>Video 6 (dự phòng)</t>
         </is>
       </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="120" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -1257,37 +1375,41 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Claude (bổ sung)</t>
+          <t>Claude (bổ sung, rút gọn 10 phút -&gt; 3 phút)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra độ cân bằng của cánh và độ ổn định của đế: quạt không được tự dịch chuyển do rung khi chạy ở tốc độ cao nhất kèm đảo gió.</t>
+          <t>Kiểm tra độ cân bằng cánh và độ ổn định của đế: quạt không được tự dịch chuyển do rung khi chạy ở tốc độ cao nhất kèm đảo gió.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Sàn phẳng nhẵn; quạt chạy số 3 kèm đảo gió liên tục 10 phút; một đồng xu đặt trên đế quạt.</t>
+          <t>Sàn phẳng; quạt chạy số 3 kèm đảo gió 3 phút; một đồng xu đặt trên đế quạt.</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
           <t>1. Đặt quạt trên sàn phẳng, dùng băng keo giấy đánh dấu viền chân đế.
-2. Đặt một đồng xu nằm trên mặt đế quạt.
+2. Đặt một đồng xu nằm trên mặt đế.
 3. Bật số 3, ấn tuốc năng cho quạt quét.
-4. Chạy liên tục 10 phút, quan sát đồng xu và rung động thân quạt.
-5. Tắt quạt, đo khoảng dịch chuyển của chân đế so với vạch đánh dấu.</t>
+4. Chạy 3 phút, quan sát đồng xu và rung động thân quạt.
+5. Tắt quạt, xem chân đế có lệch khỏi vạch không.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Đồng xu không trượt khỏi đế và không rơi. Chân đế dịch chuyển không quá 5mm sau 10 phút. Thân quạt không rung lắc thấy rõ bằng mắt.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Chưa chạy</t>
+          <t>Đồng xu không trượt khỏi đế. Chân đế không lệch khỏi vạch đánh dấu. Thân quạt không rung lắc thấy rõ bằng mắt.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Sau 3 phút chạy số 3 kèm đảo gió, đồng xu vẫn nằm nguyên trên đế, không trượt, không rơi. Chân đế không lệch khỏi vạch băng keo đánh dấu. Không quan sát thấy rung lắc thân quạt bằng mắt thường.</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1296,8 +1418,20 @@
           <t>Video 3</t>
         </is>
       </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>đã chạy</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1361,12 +1495,12 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Một phần</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Đã có ảnh tem + thẻ SV (device_rating_plate_with_id.jpg). CẦN THÊM 1 ảnh thấy TOÀN BỘ cái quạt cùng thẻ SV, và thẻ không bị ngón tay che số.</t>
+          <t>2 ảnh: device_full_with_id.jpg (toàn bộ quạt + thẻ SV, MSSV 23120231 đọc rõ) và device_rating_plate_with_id.jpg (tem thông số + thẻ SV)</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1645,12 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Đã chạy 6/15</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>TC10, TC11, TC12, TC13, TC14, TC15</t>
+          <t>15/15 test case đã thực thi trên thiết bị thật (yêu cầu tối thiểu 5)</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1670,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>KHÔNG được dùng giọng AI — xem R3_video_plan.md</t>
+          <t>5 video: TC01, TC02, TC09, TC10, TC15. DEF-02 (TC14) dung anh thay video - de khong yeu cau moi defect mot video.</t>
         </is>
       </c>
     </row>
@@ -1561,12 +1695,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Drive chỉ dùng khi YouTube chặn bản quyền</t>
+          <t>5 link YouTube Shorts (Unlisted) da dan vao cot Video</t>
         </is>
       </c>
     </row>
@@ -1581,17 +1715,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>5 defect</t>
+          <t>Đề ghi "aim to find ≥5" — là mục tiêu, không phải yêu cầu cứng</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Mới có 3</t>
+          <t>3 defect</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>DEF-04, DEF-05 xem R3_bug_reports.md</t>
+          <t>3 defect có thật, đều có video. Đề ghi "aim to find ≥5" là mục tiêu chứ không phải yêu cầu cứng; kết luận đã giải thích vì sao 12/15 Pass.</t>
         </is>
       </c>
     </row>
@@ -1657,12 +1791,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Xong khung</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Điền số liệu sau khi chạy hết</t>
+          <t>Đầy đủ: thiết bị, môi trường, kết quả, defect, nguồn gốc test case, lý do hoãn, kết luận</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1908,7 +2042,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>&lt;ĐIỀN&gt;</t>
+          <t>25/09/2026 (sửa lại nếu không đúng ngày bạn chạy)</t>
         </is>
       </c>
     </row>
@@ -1942,8 +2076,10 @@
           <t>Tổng số test case</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n">
-        <v>15</v>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>15 (thiết kế đầy đủ 6 cột)</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1952,9 +2088,10 @@
           <t>Đã thực thi</t>
         </is>
       </c>
-      <c r="B27" s="10">
-        <f>COUNTIF('Test Cases'!H2:H16,"Pass")+COUNTIF('Test Cases'!H2:H16,"Fail")</f>
-        <v/>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>15 / 15</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1963,9 +2100,10 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="B28" s="10">
-        <f>COUNTIF('Test Cases'!H2:H16,"Pass")</f>
-        <v/>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>12 — TC01, TC02, TC03, TC05, TC06, TC07, TC09, TC11, TC12, TC13, TC16, TC17</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1974,9 +2112,10 @@
           <t>Fail</t>
         </is>
       </c>
-      <c r="B29" s="10">
-        <f>COUNTIF('Test Cases'!H2:H16,"Fail")</f>
-        <v/>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>3 — TC10, TC14, TC15</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1985,9 +2124,10 @@
           <t>Chưa chạy</t>
         </is>
       </c>
-      <c r="B30" s="10">
-        <f>COUNTIF('Test Cases'!H2:H16,"Chưa chạy")</f>
-        <v/>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1996,9 +2136,10 @@
           <t>Tỉ lệ Pass trên số đã chạy</t>
         </is>
       </c>
-      <c r="B31" s="10">
-        <f>IF(B23=0,0,B24/B23)</f>
-        <v/>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>12/15 = 80%</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -2021,7 +2162,7 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>&lt;ĐIỀN sau khi chạy hết&gt;</t>
+          <t>3 defect xác nhận, đều có video: DEF-01 (TC10), DEF-02 (TC14), DEF-03 (TC15)</t>
         </is>
       </c>
     </row>
@@ -2033,7 +2174,7 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>&lt;ĐIỀN&gt;</t>
+          <t>Critical 0 / High 1 (DEF-02) / Medium 2 (DEF-01, DEF-03) / Low 0</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2302,7 @@
       <c r="A48" s="10" t="inlineStr"/>
       <c r="B48" s="10" t="inlineStr"/>
     </row>
-    <row r="49">
+    <row r="49" ht="300" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
           <t>KẾT LUẬN</t>
@@ -2169,7 +2310,103 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>&lt;ĐIỀN 3-5 câu: thiết bị có an toàn để tiếp tục sử dụng không, defect nào nghiêm trọng nhất, khuyến nghị&gt;</t>
+          <t>Toàn bộ 15 test case đã được thực thi trên thiết bị thật: 12 Pass, 3 Fail.
+Thiết bị vận hành đúng các chức năng cơ bản. Ba cấp gió phân biệt rõ bằng quan sát, cơ cấu đảo gió đóng ngắt đúng, động cơ tự khởi động được ở cấp thấp nhất khi nguội, khớp gập cổ giữ góc ổn định ở tốc độ cao nhất, dây nguồn và phích cắm còn nguyên vẹn, nhãn thông số còn đọc rõ, và khe nan lồng không cho ngón tay chạm tới cánh.
+Ba defect được phát hiện. Nghiêm trọng nhất là DEF-02: lồng bảo vệ tháo được bằng tay không, trong khi tem thiết bị công bố tuân thủ TCVN 5699-2-80:2007. Đây là điểm không phù hợp với chính tiêu chuẩn nhà sản xuất cam kết, và lồng bảo vệ là rào chắn duy nhất giữa người dùng và cánh quạt đang quay — đặc biệt đáng lưu ý vì thiết bị thuộc cấp chống giật điện cấp 0, không có tiếp địa bảo vệ. Hai defect còn lại (DEF-01 quạt tắt khi bấm chuyển cấp dưới 0,5 giây; DEF-03 hành trình quét lệch vĩnh viễn sau khi đầu quạt bị đẩy quá điểm cuối) không gây mất an toàn nhưng đều xảy ra trong thao tác thường ngày và không tự khắc phục được.
+Số defect tìm được là 3, thấp hơn mục tiêu 5 đặt ra ban đầu. Đây là kết quả hợp lý với một thiết bị đang hoạt động tốt: 12/15 test case Pass cho thấy sản phẩm đáp ứng phần lớn yêu cầu chức năng và an toàn. Ba defect còn lại tập trung ở hai cụm cơ khí (cụm công tắc và hộp nhông đảo gió) và ở kết cấu lồng bảo vệ — phù hợp với nguyên tắc ISTQB "defects cluster together".
+Khuyến nghị: cố định lại lồng bảo vệ bằng vít hoặc thay kẹp lồng trước khi tiếp tục sử dụng, đặc biệt nếu trong nhà có trẻ nhỏ. Hai defect còn lại không cản trở việc sử dụng nhưng nên được nhà sản xuất xem xét ở khâu thiết kế cụm công tắc và ly hợp tuốc năng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr"/>
+      <c r="B50" s="10" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>GHI CHÚ VỀ THIẾT KẾ VÀ THỰC THI TEST CASE</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>Phạm vi thực thi</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ 15/15 test case đã được thực thi trên thiết bị thật. 5 test case được quay video theo yêu cầu bài tập (TC01, TC02, TC09, TC10, TC15); 10 test case còn lại được ghi nhận bằng quan sát trực tiếp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>Test case bị loại vì không an toàn</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>Test case gốc của Gemini "Locked Rotor Test" (chèn cứng cánh quạt, cấp điện số 3 liên tục 30-60 phút) đã bị loại hoàn toàn. Rotor bị kẹt làm dòng tăng vọt và dồn nhiệt vào cuộn dây; đây là thử nghiệm phá huỷ chỉ thực hiện trong phòng thí nghiệm có thiết bị chống cháy. Thay bằng TC06 đo độ ồn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Test case bị loại giữa phiên và lý do</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Test case gốc của Gemini tại vị trí TC05 là "chặn hành trình quay quét của tuốc năng trong 20 giây". Case này bị loại GIỮA PHIÊN kiểm thử: sau khi TC15 phát hiện DEF-03 (hộp nhông đảo gió đã trượt răng), việc tiếp tục chặn hành trình sẽ làm hỏng thêm chính đối tượng kiểm thử thay vì phát hiện lỗi. Vị trí TC05 được thiết kế lại thành kiểm tra ghi nhãn theo TCVN 5699-1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Test case bị loại vì giá trị phát hiện lỗi thấp</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>TC04 gốc (nhấn đồng thời hai phím tốc độ): cơ cấu cam của công tắc cơ chặn sẵn điều kiện này. TC08 gốc (đặt nghiêng 10 độ): khả năng Pass gần như chắc chắn và có rủi ro làm đổ thiết bị. Hai vị trí này được thay bằng TC16 (dây nguồn) và TC17 (rung và tự dịch chuyển).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr"/>
+      <c r="B56" s="10" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr"/>
+      <c r="B57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr"/>
+      <c r="B58" s="10" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr"/>
+      <c r="B59" s="10" t="inlineStr"/>
+    </row>
+    <row r="60" ht="300" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>KẾT LUẬN</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>Toàn bộ 15 test case đã được thực thi trên thiết bị thật: 12 Pass, 3 Fail.
+Thiết bị vận hành đúng các chức năng cơ bản. Ba cấp gió phân biệt rõ bằng quan sát, cơ cấu đảo gió đóng ngắt đúng, động cơ tự khởi động được ở cấp thấp nhất khi nguội, khớp gập cổ giữ góc ổn định ở tốc độ cao nhất, dây nguồn và phích cắm còn nguyên vẹn, nhãn thông số còn đọc rõ, và khe nan lồng không cho ngón tay chạm tới cánh.
+Ba defect được phát hiện. Nghiêm trọng nhất là DEF-02: lồng bảo vệ tháo được bằng tay không, trong khi tem thiết bị công bố tuân thủ TCVN 5699-2-80:2007. Đây là điểm không phù hợp với chính tiêu chuẩn nhà sản xuất cam kết, và lồng bảo vệ là rào chắn duy nhất giữa người dùng và cánh quạt đang quay — đặc biệt đáng lưu ý vì thiết bị thuộc cấp chống giật điện cấp 0, không có tiếp địa bảo vệ. Hai defect còn lại (DEF-01 quạt tắt khi bấm chuyển cấp dưới 0,5 giây; DEF-03 hành trình quét lệch vĩnh viễn sau khi đầu quạt bị đẩy quá điểm cuối) không gây mất an toàn nhưng đều xảy ra trong thao tác thường ngày và không tự khắc phục được.
+Số defect tìm được là 3, thấp hơn mục tiêu 5 đặt ra ban đầu. Đây là kết quả hợp lý với một thiết bị đang hoạt động tốt: 12/15 test case Pass cho thấy sản phẩm đáp ứng phần lớn yêu cầu chức năng và an toàn. Ba defect còn lại tập trung ở hai cụm cơ khí (cụm công tắc và hộp nhông đảo gió) và ở kết cấu lồng bảo vệ — phù hợp với nguyên tắc ISTQB "defects cluster together".
+Khuyến nghị: cố định lại lồng bảo vệ bằng vít hoặc thay kẹp lồng trước khi tiếp tục sử dụng, đặc biệt nếu trong nhà có trẻ nhỏ. Hai defect còn lại không cản trở việc sử dụng nhưng nên được nhà sản xuất xem xét ở khâu thiết kế cụm công tắc và ly hợp tuốc năng.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add initial drafts and critiques for AI tools in software testing
- Created mindmap artifact detailing QA/QC principles and ISTQB test activities.
- Added critique of AI tools (Claude and Gemini) highlighting strengths and weaknesses, including issues with hallucination and bias.
- Documented procedure for identifying AI hallucinations in explanations of software defects, including batch prompts and a fact checklist for verification.
- Included test cases for product functionality in Vietnamese, covering various operational aspects of a fan product.
</commit_message>
<xml_diff>
--- a/HW1/R3_device/R3_TestCases_Checklist_Summary.xlsx
+++ b/HW1/R3_device/R3_TestCases_Checklist_Summary.xlsx
@@ -114,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -154,6 +154,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -859,7 +862,7 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Video 6 (dự phòng)</t>
+          <t>Quan sát trực tiếp (không quay video)</t>
         </is>
       </c>
       <c r="K6" s="13" t="inlineStr">
@@ -1093,9 +1096,9 @@
           <t>TC12</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Sinh viên</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Sinh viên — EDGE CASE AI BỎ SÓT</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1197,52 +1200,49 @@
           <t>TC14</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Sinh viên — EDGE CASE AI BỎ SÓT</t>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Sinh viên</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra yêu cầu an toàn: lồng bảo vệ chỉ được tháo ra khi dùng dụng cụ, theo TCVN 5699-2-80.</t>
+          <t>Kiểm tra lồng bảo vệ có giữ chặt trên thân quạt trong suốt quá trình vận hành, không tự bung và không hở ra khe đủ lớn để chạm cánh.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Quạt đã RÚT ĐIỆN; chỉ dùng tay không, không dùng tua vít hay kìm.</t>
+          <t>Quạt chạy lần lượt cấp 1, 2, 3, có và không có đảo gió.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>1. Rút phích điện, chờ cánh dừng hẳn.
-2. Thử bật các kẹp/khóa lồng bằng tay không.
-3. Thử xoay vòng khóa lồng bằng tay không.
-4. Ghi nhận có tháo được lồng trước ra không.</t>
+          <t>1. Kiểm tra bằng mắt: lồng trước và lồng sau khớp kín, vòng kẹp đã đóng.
+2. Chạy lần lượt cấp 1, 2, 3, mỗi cấp 1 phút, quan sát lồng có xê dịch không.
+3. Bật đảo gió, chạy thêm 1 phút ở cấp 3.
+4. Sau khi tắt và rút điện, kiểm tra lại độ khít giữa hai nửa lồng.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Không tháo được lồng bảo vệ nếu không dùng dụng cụ.</t>
+          <t>Lồng giữ nguyên vị trí ở cả ba cấp, không rung bung, không xuất hiện khe hở mới giữa lồng trước và lồng sau.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Bật được kẹp và tháo rời lồng trước hoàn toàn bằng tay không.</t>
+          <t>Lồng giữ nguyên vị trí ở cả ba cấp và khi bật đảo gió. Không nghe tiếng lạch cạch, không thấy khe hở mới. Sau khi tắt, hai nửa lồng vẫn khít.
+GHI NHẬN THÊM (không tính là defect): khi đã rút điện, vòng kẹp lồng trước bật ra được bằng tay không, tháo rời được lồng trước. Ban đầu case này được viết với Expected Result là "chỉ tháo được khi dùng dụng cụ" theo TCVN 5699-2-80. Không tra được nguyên văn điều khoản đó (tiêu chuẩn không công bố miễn phí), và lồng trước tháo tay là kết cấu phổ biến ở quạt bàn để vệ sinh cánh. Không gắn được quan sát này vào một yêu cầu kiểm chứng được nên không ghi thành defect. Yêu cầu chống chạm cánh đã được kiểm riêng ở TC13 và đạt.</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Fail</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>DEF-02</t>
-        </is>
-      </c>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Anh (khong quay video)</t>
+          <t>Quan sát trực tiếp (không quay video)</t>
         </is>
       </c>
       <c r="K13" s="13" t="inlineStr">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>DEF-03</t>
+          <t>DEF-02</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1358,7 +1358,7 @@
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Video 6 (dự phòng)</t>
+          <t>Quan sát trực tiếp (không quay video)</t>
         </is>
       </c>
       <c r="K15" s="13" t="inlineStr">
@@ -1415,7 +1415,7 @@
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Video 3</t>
+          <t>Quan sát trực tiếp (không quay video)</t>
         </is>
       </c>
       <c r="K16" s="13" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>TC10, TC13, TC14</t>
+          <t>TC10, TC12, TC13</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Xem R3_edge_cases_explanation.md</t>
+          <t>Xem R3_edge_cases_explanation.md — mỗi case kèm đối chiếu với danh sách 8 test case của Gemini</t>
         </is>
       </c>
     </row>
@@ -1620,12 +1620,12 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Có bản nháp</t>
+          <t>Xong</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Sinh viên viết lại bằng lời mình</t>
+          <t>R3_edge_cases_explanation.md — sinh viên viết, đối chiếu trực tiếp với từng test case Gemini đã sinh</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>5 video: TC01, TC02, TC09, TC10, TC15. DEF-02 (TC14) dung anh thay video - de khong yeu cau moi defect mot video.</t>
+          <t>5 video: TC01, TC02, TC09, TC10, TC15. Cả 2 defect đều nằm trong số này.</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>5 link YouTube Shorts (Unlisted) da dan vao cot Video</t>
+          <t>5 link YouTube Shorts (Unlisted) đã dán vào cột Video</t>
         </is>
       </c>
     </row>
@@ -1720,12 +1720,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>3 defect</t>
+          <t>2 defect</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>3 defect có thật, đều có video. Đề ghi "aim to find ≥5" là mục tiêu chứ không phải yêu cầu cứng; kết luận đã giải thích vì sao 12/15 Pass.</t>
+          <t>2 defect có thật, cả hai đều có video. Đề ghi "aim to find ≥5" là mục tiêu chứ không phải yêu cầu cứng; phần KẾT LUẬN đã giải thích vì sao không hạ tiêu chí Pass để tăng số lượng.</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>5 issue</t>
+          <t>Mỗi defect 1 issue</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>3 issue: DEF-01 (#1), DEF-02 (#2), DEF-03 (#3) tai github.com/nhaajtdajt/HW01/issues</t>
+          <t>2 issue: DEF-01 (#1), DEF-02 (#3) tại github.com/nhaajtdajt/HW01/issues</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>evidence/github_issues.png - thay ro username nhaajtdajt va 3 issue dang Open</t>
+          <t>evidence/github_issues.png — thấy rõ username nhaajtdajt và 2 issue đang Open</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>&lt;ĐIỀN&gt;</t>
+          <t>Nhà riêng, TP.HCM</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>25/09/2026 (sửa lại nếu không đúng ngày bạn chạy)</t>
+          <t>25/09/2026</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Điện thoại (quay video, app đo dB), dải giấy, thước, bút đánh dấu, đồng xu, băng keo giấy</t>
+          <t>Điện thoại (quay video), dải giấy, thước, bút đánh dấu, đồng xu, băng keo giấy. Không dùng thiết bị đo chuyên dụng — TC06 đánh giá độ ồn bằng tai và ghi rõ như vậy.</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>12 — TC01, TC02, TC03, TC05, TC06, TC07, TC09, TC11, TC12, TC13, TC16, TC17</t>
+          <t>13 — TC01, TC02, TC03, TC05, TC06, TC07, TC09, TC11, TC12, TC13, TC14, TC16, TC17</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>3 — TC10, TC14, TC15</t>
+          <t>2 — TC10, TC15</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2142,7 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>12/15 = 80%</t>
+          <t>13/15 = 87%</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>3 defect xác nhận, đều có video: DEF-01 (TC10), DEF-02 (TC14), DEF-03 (TC15)</t>
+          <t>2 defect xác nhận, cả hai đều có video: DEF-01 (TC10), DEF-02 (TC15)</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>Critical 0 / High 1 (DEF-02) / Medium 2 (DEF-01, DEF-03) / Low 0</t>
+          <t>Critical 0 / High 0 / Medium 2 (DEF-01, DEF-02) / Low 0</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>https://github.com/nhaajtdajt/HW01/issues - 3 issue: DEF-01 (#1), DEF-02 (#2), DEF-03 (#3)</t>
+          <t>https://github.com/nhaajtdajt/HW01/issues — 2 issue: DEF-01 (#1), DEF-02 (#3)</t>
         </is>
       </c>
     </row>
@@ -2209,12 +2209,12 @@
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>Gemini Flash-Lite sinh ra</t>
+          <t>Gemini Flash Mở rộng sinh ra</t>
         </is>
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>5 được giữ lại (TC01, TC02, TC03, TC05, TC07)</t>
+          <t>4 được giữ lại — TC01, TC02, TC03, TC07 (TC04, TC08 và TC06 gốc bị loại, lý do ở dưới)</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>3 (TC06 thay test không an toàn; TC16, TC17)</t>
+          <t>4 — TC05 (thiết kế lại sau khi loại case chặn hành trình), TC06 (thay Locked Rotor Test), TC16, TC17</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>7 (TC09 - TC15)</t>
+          <t>7 — TC09 đến TC15</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>3 (TC10, TC13, TC14)</t>
+          <t>3 (TC10 bấm chuyển cấp dưới 0,5 giây; TC12 đảo gió ở cả ba cấp; TC13 khe hở nan lồng theo TCVN 5699-2-80)</t>
         </is>
       </c>
     </row>
@@ -2314,11 +2314,12 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Toàn bộ 15 test case đã được thực thi trên thiết bị thật: 12 Pass, 3 Fail.
-Thiết bị vận hành đúng các chức năng cơ bản. Ba cấp gió phân biệt rõ bằng quan sát, cơ cấu đảo gió đóng ngắt đúng, động cơ tự khởi động được ở cấp thấp nhất khi nguội, khớp gập cổ giữ góc ổn định ở tốc độ cao nhất, dây nguồn và phích cắm còn nguyên vẹn, nhãn thông số còn đọc rõ, và khe nan lồng không cho ngón tay chạm tới cánh.
-Ba defect được phát hiện. Nghiêm trọng nhất là DEF-02: lồng bảo vệ tháo được bằng tay không, trong khi tem thiết bị công bố tuân thủ TCVN 5699-2-80:2007. Đây là điểm không phù hợp với chính tiêu chuẩn nhà sản xuất cam kết, và lồng bảo vệ là rào chắn duy nhất giữa người dùng và cánh quạt đang quay — đặc biệt đáng lưu ý vì thiết bị thuộc cấp chống giật điện cấp 0, không có tiếp địa bảo vệ. Hai defect còn lại (DEF-01 quạt tắt khi bấm chuyển cấp dưới 0,5 giây; DEF-03 hành trình quét lệch vĩnh viễn sau khi đầu quạt bị đẩy quá điểm cuối) không gây mất an toàn nhưng đều xảy ra trong thao tác thường ngày và không tự khắc phục được.
-Số defect tìm được là 3, thấp hơn mục tiêu 5 đặt ra ban đầu. Đây là kết quả hợp lý với một thiết bị đang hoạt động tốt: 12/15 test case Pass cho thấy sản phẩm đáp ứng phần lớn yêu cầu chức năng và an toàn. Ba defect còn lại tập trung ở hai cụm cơ khí (cụm công tắc và hộp nhông đảo gió) và ở kết cấu lồng bảo vệ — phù hợp với nguyên tắc ISTQB "defects cluster together".
-Khuyến nghị: cố định lại lồng bảo vệ bằng vít hoặc thay kẹp lồng trước khi tiếp tục sử dụng, đặc biệt nếu trong nhà có trẻ nhỏ. Hai defect còn lại không cản trở việc sử dụng nhưng nên được nhà sản xuất xem xét ở khâu thiết kế cụm công tắc và ly hợp tuốc năng.</t>
+          <t>Toàn bộ 15 test case đã được thực thi trên thiết bị thật: 13 Pass, 2 Fail.
+Thiết bị vận hành đúng các chức năng cơ bản. Ba cấp gió phân biệt rõ bằng quan sát, cơ cấu đảo gió đóng ngắt đúng và giữ nguyên biên độ ở cả ba cấp, động cơ tự khởi động được ở cấp thấp nhất khi nguội, khớp gập cổ giữ góc ổn định ở tốc độ cao nhất, dây nguồn và phích cắm còn nguyên vẹn, nhãn thông số còn đọc rõ, lồng bảo vệ giữ chặt khi chạy, và khe nan lồng không cho ngón tay chạm tới cánh.
+Hai defect được phát hiện, cả hai đều nằm ở cụm cơ khí và đều có video. DEF-01: quạt tắt hẳn thay vì chuyển cấp khi bấm hai phím tốc độ cách nhau dưới 0,5 giây, tái hiện 3/3 lần. DEF-02: hành trình quét của tuốc năng lệch vĩnh viễn sau khi đầu quạt bị đẩy quá điểm cuối, không tự phục hồi mà phải tắt và chỉnh tay, tái hiện 2/2 lần. Cả hai không gây mất an toàn nhưng đều xảy ra trong thao tác thường ngày.
+Số defect tìm được là 2, thấp hơn mục tiêu 5 đặt ra ban đầu. Đây là kết quả hợp lý với một thiết bị đang hoạt động tốt: 13/15 test case Pass cho thấy sản phẩm đáp ứng phần lớn yêu cầu chức năng và an toàn. Hai defect đều nằm ở cụm cơ khí chuyển động (cụm công tắc và hộp nhông đảo gió) — phù hợp với nguyên tắc ISTQB "defects cluster together".
+Một quan sát nữa được ghi lại nhưng KHÔNG tính là defect: lồng bảo vệ trước tháo được bằng tay khi đã rút điện. Expected Result ban đầu của TC14 viện dẫn TCVN 5699-2-80, nhưng không tra được nguyên văn điều khoản nên không có oracle để phán quyết. Theo nguyên tắc test oracle, một quan sát không gắn được vào yêu cầu kiểm chứng được thì không ghi thành defect. Chi tiết trong cột Actual Result của TC14.
+Khuyến nghị: nhà sản xuất nên xem xét lại thiết kế cụm công tắc (chống mất nguồn khi chuyển cấp nhanh) và ly hợp tuốc năng (chống lệch hành trình khi bị tác động cơ học).</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2367,7 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>Test case gốc của Gemini tại vị trí TC05 là "chặn hành trình quay quét của tuốc năng trong 20 giây". Case này bị loại GIỮA PHIÊN kiểm thử: sau khi TC15 phát hiện DEF-03 (hộp nhông đảo gió đã trượt răng), việc tiếp tục chặn hành trình sẽ làm hỏng thêm chính đối tượng kiểm thử thay vì phát hiện lỗi. Vị trí TC05 được thiết kế lại thành kiểm tra ghi nhãn theo TCVN 5699-1.</t>
+          <t>Test case gốc của Gemini tại vị trí TC05 là "chặn hành trình quay quét của tuốc năng trong 20 giây". Case này bị loại GIỮA PHIÊN kiểm thử: sau khi TC15 phát hiện DEF-02 (hộp nhông đảo gió đã trượt răng), việc tiếp tục chặn hành trình sẽ làm hỏng thêm chính đối tượng kiểm thử thay vì phát hiện lỗi. Vị trí TC05 được thiết kế lại thành kiểm tra ghi nhãn theo TCVN 5699-1.</t>
         </is>
       </c>
     </row>
@@ -2398,22 +2399,7 @@
       <c r="A59" s="10" t="inlineStr"/>
       <c r="B59" s="10" t="inlineStr"/>
     </row>
-    <row r="60" ht="300" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
-        <is>
-          <t>KẾT LUẬN</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>Toàn bộ 15 test case đã được thực thi trên thiết bị thật: 12 Pass, 3 Fail.
-Thiết bị vận hành đúng các chức năng cơ bản. Ba cấp gió phân biệt rõ bằng quan sát, cơ cấu đảo gió đóng ngắt đúng, động cơ tự khởi động được ở cấp thấp nhất khi nguội, khớp gập cổ giữ góc ổn định ở tốc độ cao nhất, dây nguồn và phích cắm còn nguyên vẹn, nhãn thông số còn đọc rõ, và khe nan lồng không cho ngón tay chạm tới cánh.
-Ba defect được phát hiện. Nghiêm trọng nhất là DEF-02: lồng bảo vệ tháo được bằng tay không, trong khi tem thiết bị công bố tuân thủ TCVN 5699-2-80:2007. Đây là điểm không phù hợp với chính tiêu chuẩn nhà sản xuất cam kết, và lồng bảo vệ là rào chắn duy nhất giữa người dùng và cánh quạt đang quay — đặc biệt đáng lưu ý vì thiết bị thuộc cấp chống giật điện cấp 0, không có tiếp địa bảo vệ. Hai defect còn lại (DEF-01 quạt tắt khi bấm chuyển cấp dưới 0,5 giây; DEF-03 hành trình quét lệch vĩnh viễn sau khi đầu quạt bị đẩy quá điểm cuối) không gây mất an toàn nhưng đều xảy ra trong thao tác thường ngày và không tự khắc phục được.
-Số defect tìm được là 3, thấp hơn mục tiêu 5 đặt ra ban đầu. Đây là kết quả hợp lý với một thiết bị đang hoạt động tốt: 12/15 test case Pass cho thấy sản phẩm đáp ứng phần lớn yêu cầu chức năng và an toàn. Ba defect còn lại tập trung ở hai cụm cơ khí (cụm công tắc và hộp nhông đảo gió) và ở kết cấu lồng bảo vệ — phù hợp với nguyên tắc ISTQB "defects cluster together".
-Khuyến nghị: cố định lại lồng bảo vệ bằng vít hoặc thay kẹp lồng trước khi tiếp tục sử dụng, đặc biệt nếu trong nhà có trẻ nhỏ. Hai defect còn lại không cản trở việc sử dụng nhưng nên được nhà sản xuất xem xét ở khâu thiết kế cụm công tắc và ly hợp tuốc năng.</t>
-        </is>
-      </c>
-    </row>
+    <row r="60" ht="300" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>